<commit_message>
Added RDF data schemes and fixed visual schemes for geography-table01-04
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/geography-table04.xlsx
+++ b/sources/table_normalization/xlsx/geography-table04.xlsx
@@ -425,7 +425,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -486,61 +486,49 @@
     <xf numFmtId="2" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -849,7 +837,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -883,159 +871,159 @@
       <c r="E1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="22" t="s">
+      <c r="G1" s="33"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="22" t="s">
+      <c r="J1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="19" t="s">
+      <c r="K1" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="24" t="s">
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
+      <c r="R1" s="34"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="22" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="52">
       <c r="A2" s="16"/>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="26"/>
       <c r="D2" s="18" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="18"/>
-      <c r="F2" s="26" t="s">
+      <c r="F2" s="24" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="H2" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22" t="s">
+      <c r="I2" s="20"/>
+      <c r="J2" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="30" t="s">
+      <c r="K2" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="L2" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="M2" s="22" t="s">
+      <c r="M2" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="22" t="s">
+      <c r="N2" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="22" t="s">
+      <c r="O2" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="P2" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="25" t="s">
+      <c r="Q2" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="31" t="s">
+      <c r="R2" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="31" t="s">
+      <c r="S2" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="T2" s="24" t="s">
+      <c r="T2" s="22" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="26">
       <c r="A3" s="16"/>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="26"/>
       <c r="D3" s="18" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="18"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="22" t="s">
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="J3" s="22" t="s">
+      <c r="J3" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="32"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="33"/>
-      <c r="R3" s="33"/>
-      <c r="S3" s="33"/>
-      <c r="T3" s="25"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="30"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="31"/>
+      <c r="T3" s="23"/>
     </row>
     <row r="4" spans="1:20" ht="39.5" thickBot="1">
       <c r="A4" s="16"/>
-      <c r="B4" s="27"/>
-      <c r="C4" s="28"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="26"/>
       <c r="D4" s="18" t="s">
         <v>73</v>
       </c>
       <c r="E4" s="18"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="22" t="s">
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="J4" s="22" t="s">
+      <c r="J4" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="34" t="s">
+      <c r="K4" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="35" t="s">
+      <c r="L4" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="35" t="s">
+      <c r="M4" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="35" t="s">
+      <c r="N4" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="35" t="s">
+      <c r="O4" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="36" t="s">
+      <c r="P4" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="Q4" s="37" t="s">
+      <c r="Q4" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="38" t="s">
+      <c r="R4" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="31"/>
-      <c r="T4" s="25"/>
+      <c r="S4" s="29"/>
+      <c r="T4" s="23"/>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="4">

</xml_diff>